<commit_message>
timetable: import every bus.jeju.go.kr timetable (2026-10-19) {'parsed': 201, 'source_conflict': 30, 'no_timetable': 4}
Workflow run 39168127136.
</commit_message>
<xml_diff>
--- a/fixtures/jeju/timetables/bis/raw/405001.xlsx
+++ b/fixtures/jeju/timetables/bis/raw/405001.xlsx
@@ -6,8 +6,8 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="101 공항-조천-김녕-성산-남원" r:id="rId3" sheetId="1"/>
-    <sheet name="101 남원-성산-김녕-조천-공항" r:id="rId4" sheetId="2"/>
+    <sheet name="101 남원-성산-김녕-조천-공항" r:id="rId3" sheetId="1"/>
+    <sheet name="101 공항-조천-김녕-성산-남원" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
@@ -18,37 +18,568 @@
     <t>구분</t>
   </si>
   <si>
-    <t>공항</t>
+    <t>남원</t>
+  </si>
+  <si>
+    <t>표선</t>
+  </si>
+  <si>
+    <t>고성</t>
+  </si>
+  <si>
+    <t>성산</t>
+  </si>
+  <si>
+    <t>세화</t>
+  </si>
+  <si>
+    <t>김녕</t>
+  </si>
+  <si>
+    <t>함덕</t>
   </si>
   <si>
     <t>제주
 버스터미널</t>
   </si>
   <si>
-    <t>함덕</t>
-  </si>
-  <si>
-    <t>김녕</t>
-  </si>
-  <si>
-    <t>세화</t>
-  </si>
-  <si>
-    <t>성산</t>
-  </si>
-  <si>
-    <t>고성</t>
-  </si>
-  <si>
-    <t>표선</t>
-  </si>
-  <si>
-    <t>남원</t>
+    <t>공항</t>
   </si>
   <si>
     <t>X</t>
   </si>
   <si>
+    <t>06:00</t>
+  </si>
+  <si>
+    <t>06:18</t>
+  </si>
+  <si>
+    <t>06:36</t>
+  </si>
+  <si>
+    <t>06:50</t>
+  </si>
+  <si>
+    <t>07:26</t>
+  </si>
+  <si>
+    <t>07:34</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t>07:18</t>
+  </si>
+  <si>
+    <t>07:36</t>
+  </si>
+  <si>
+    <t>07:50</t>
+  </si>
+  <si>
+    <t>08:26</t>
+  </si>
+  <si>
+    <t>08:34</t>
+  </si>
+  <si>
+    <t>07:09</t>
+  </si>
+  <si>
+    <t>07:46</t>
+  </si>
+  <si>
+    <t>07:53</t>
+  </si>
+  <si>
+    <t>08:11</t>
+  </si>
+  <si>
+    <t>08:29</t>
+  </si>
+  <si>
+    <t>08:43</t>
+  </si>
+  <si>
+    <t>09:19</t>
+  </si>
+  <si>
+    <t>09:27</t>
+  </si>
+  <si>
+    <t>08:14</t>
+  </si>
+  <si>
+    <t>08:31</t>
+  </si>
+  <si>
+    <t>08:51</t>
+  </si>
+  <si>
+    <t>08:58</t>
+  </si>
+  <si>
+    <t>09:16</t>
+  </si>
+  <si>
+    <t>09:34</t>
+  </si>
+  <si>
+    <t>09:48</t>
+  </si>
+  <si>
+    <t>10:24</t>
+  </si>
+  <si>
+    <t>10:32</t>
+  </si>
+  <si>
+    <t>09:10</t>
+  </si>
+  <si>
+    <t>09:47</t>
+  </si>
+  <si>
+    <t>09:54</t>
+  </si>
+  <si>
+    <t>10:12</t>
+  </si>
+  <si>
+    <t>10:30</t>
+  </si>
+  <si>
+    <t>10:44</t>
+  </si>
+  <si>
+    <t>11:20</t>
+  </si>
+  <si>
+    <t>11:28</t>
+  </si>
+  <si>
+    <t>10:04</t>
+  </si>
+  <si>
+    <t>10:21</t>
+  </si>
+  <si>
+    <t>10:41</t>
+  </si>
+  <si>
+    <t>10:48</t>
+  </si>
+  <si>
+    <t>11:06</t>
+  </si>
+  <si>
+    <t>11:24</t>
+  </si>
+  <si>
+    <t>11:38</t>
+  </si>
+  <si>
+    <t>12:14</t>
+  </si>
+  <si>
+    <t>12:22</t>
+  </si>
+  <si>
+    <t>10:54</t>
+  </si>
+  <si>
+    <t>11:11</t>
+  </si>
+  <si>
+    <t>11:31</t>
+  </si>
+  <si>
+    <t>11:56</t>
+  </si>
+  <si>
+    <t>12:28</t>
+  </si>
+  <si>
+    <t>13:04</t>
+  </si>
+  <si>
+    <t>13:12</t>
+  </si>
+  <si>
+    <t>11:34</t>
+  </si>
+  <si>
+    <t>11:51</t>
+  </si>
+  <si>
+    <t>12:11</t>
+  </si>
+  <si>
+    <t>12:18</t>
+  </si>
+  <si>
+    <t>12:36</t>
+  </si>
+  <si>
+    <t>12:54</t>
+  </si>
+  <si>
+    <t>13:08</t>
+  </si>
+  <si>
+    <t>13:44</t>
+  </si>
+  <si>
+    <t>13:52</t>
+  </si>
+  <si>
+    <t>12:24</t>
+  </si>
+  <si>
+    <t>12:41</t>
+  </si>
+  <si>
+    <t>13:01</t>
+  </si>
+  <si>
+    <t>13:26</t>
+  </si>
+  <si>
+    <t>13:58</t>
+  </si>
+  <si>
+    <t>14:34</t>
+  </si>
+  <si>
+    <t>14:42</t>
+  </si>
+  <si>
+    <t>13:24</t>
+  </si>
+  <si>
+    <t>13:41</t>
+  </si>
+  <si>
+    <t>14:01</t>
+  </si>
+  <si>
+    <t>14:08</t>
+  </si>
+  <si>
+    <t>14:26</t>
+  </si>
+  <si>
+    <t>14:44</t>
+  </si>
+  <si>
+    <t>14:58</t>
+  </si>
+  <si>
+    <t>15:34</t>
+  </si>
+  <si>
+    <t>15:42</t>
+  </si>
+  <si>
+    <t>14:09</t>
+  </si>
+  <si>
+    <t>14:46</t>
+  </si>
+  <si>
+    <t>14:53</t>
+  </si>
+  <si>
+    <t>15:11</t>
+  </si>
+  <si>
+    <t>15:29</t>
+  </si>
+  <si>
+    <t>15:43</t>
+  </si>
+  <si>
+    <t>16:19</t>
+  </si>
+  <si>
+    <t>16:27</t>
+  </si>
+  <si>
+    <t>14:54</t>
+  </si>
+  <si>
+    <t>15:31</t>
+  </si>
+  <si>
+    <t>15:38</t>
+  </si>
+  <si>
+    <t>15:56</t>
+  </si>
+  <si>
+    <t>16:14</t>
+  </si>
+  <si>
+    <t>16:28</t>
+  </si>
+  <si>
+    <t>17:04</t>
+  </si>
+  <si>
+    <t>17:12</t>
+  </si>
+  <si>
+    <t>15:49</t>
+  </si>
+  <si>
+    <t>16:06</t>
+  </si>
+  <si>
+    <t>16:26</t>
+  </si>
+  <si>
+    <t>16:33</t>
+  </si>
+  <si>
+    <t>16:51</t>
+  </si>
+  <si>
+    <t>17:09</t>
+  </si>
+  <si>
+    <t>17:23</t>
+  </si>
+  <si>
+    <t>17:59</t>
+  </si>
+  <si>
+    <t>18:07</t>
+  </si>
+  <si>
+    <t>16:34</t>
+  </si>
+  <si>
+    <t>17:11</t>
+  </si>
+  <si>
+    <t>17:18</t>
+  </si>
+  <si>
+    <t>17:36</t>
+  </si>
+  <si>
+    <t>17:54</t>
+  </si>
+  <si>
+    <t>18:08</t>
+  </si>
+  <si>
+    <t>18:44</t>
+  </si>
+  <si>
+    <t>18:52</t>
+  </si>
+  <si>
+    <t>17:29</t>
+  </si>
+  <si>
+    <t>17:46</t>
+  </si>
+  <si>
+    <t>18:06</t>
+  </si>
+  <si>
+    <t>18:13</t>
+  </si>
+  <si>
+    <t>18:31</t>
+  </si>
+  <si>
+    <t>18:49</t>
+  </si>
+  <si>
+    <t>19:03</t>
+  </si>
+  <si>
+    <t>19:39</t>
+  </si>
+  <si>
+    <t>19:47</t>
+  </si>
+  <si>
+    <t>18:14</t>
+  </si>
+  <si>
+    <t>18:51</t>
+  </si>
+  <si>
+    <t>18:58</t>
+  </si>
+  <si>
+    <t>19:16</t>
+  </si>
+  <si>
+    <t>19:34</t>
+  </si>
+  <si>
+    <t>19:48</t>
+  </si>
+  <si>
+    <t>20:24</t>
+  </si>
+  <si>
+    <t>20:32</t>
+  </si>
+  <si>
+    <t>19:09</t>
+  </si>
+  <si>
+    <t>19:26</t>
+  </si>
+  <si>
+    <t>19:46</t>
+  </si>
+  <si>
+    <t>19:53</t>
+  </si>
+  <si>
+    <t>20:11</t>
+  </si>
+  <si>
+    <t>20:29</t>
+  </si>
+  <si>
+    <t>20:43</t>
+  </si>
+  <si>
+    <t>21:19</t>
+  </si>
+  <si>
+    <t>21:27</t>
+  </si>
+  <si>
+    <t>19:44</t>
+  </si>
+  <si>
+    <t>20:01</t>
+  </si>
+  <si>
+    <t>20:21</t>
+  </si>
+  <si>
+    <t>20:28</t>
+  </si>
+  <si>
+    <t>20:46</t>
+  </si>
+  <si>
+    <t>21:04</t>
+  </si>
+  <si>
+    <t>21:18</t>
+  </si>
+  <si>
+    <t>21:54</t>
+  </si>
+  <si>
+    <t>22:02</t>
+  </si>
+  <si>
+    <t>20:14</t>
+  </si>
+  <si>
+    <t>20:31</t>
+  </si>
+  <si>
+    <t>20:51</t>
+  </si>
+  <si>
+    <t>20:58</t>
+  </si>
+  <si>
+    <t>21:16</t>
+  </si>
+  <si>
+    <t>21:34</t>
+  </si>
+  <si>
+    <t>21:48</t>
+  </si>
+  <si>
+    <t>22:24</t>
+  </si>
+  <si>
+    <t>22:32</t>
+  </si>
+  <si>
+    <t>20:44</t>
+  </si>
+  <si>
+    <t>21:01</t>
+  </si>
+  <si>
+    <t>21:21</t>
+  </si>
+  <si>
+    <t>21:28</t>
+  </si>
+  <si>
+    <t>21:46</t>
+  </si>
+  <si>
+    <t>22:04</t>
+  </si>
+  <si>
+    <t>22:18</t>
+  </si>
+  <si>
+    <t>22:54</t>
+  </si>
+  <si>
+    <t>23:02</t>
+  </si>
+  <si>
+    <t>21:14</t>
+  </si>
+  <si>
+    <t>21:31</t>
+  </si>
+  <si>
+    <t>21:51</t>
+  </si>
+  <si>
+    <t>21:58</t>
+  </si>
+  <si>
+    <t>21:44</t>
+  </si>
+  <si>
+    <t>22:01</t>
+  </si>
+  <si>
+    <t>22:21</t>
+  </si>
+  <si>
+    <t>22:28</t>
+  </si>
+  <si>
+    <t>101번</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 남원읍사무소-표선리사무소-신산리-고성리-성산일출봉입구-성산항입구-성산고등학교-세화고등학교-세화리-용암해수단지-월정리-김녕초등학교-함덕해수욕장-함덕고등학교-조천리사무소-신촌초등학교-삼양동주민센터-화북남문-오현중·고등학교-천수동-동광양-제주버스터미널-공항</t>
+  </si>
+  <si>
+    <t>남원 →일주동로 → 공항</t>
+  </si>
+  <si>
+    <t>첫차(성산일출봉 출발) 6:00, 막차 21:44, 배차간격 28분~43분, 금남여객(064-753-4423)</t>
+  </si>
+  <si>
+    <t>(시행일 : 2024.8.15.)</t>
+  </si>
+  <si>
     <t>06:05</t>
   </si>
   <si>
@@ -85,12 +616,6 @@
     <t>07:28</t>
   </si>
   <si>
-    <t>07:46</t>
-  </si>
-  <si>
-    <t>07:53</t>
-  </si>
-  <si>
     <t>08:13</t>
   </si>
   <si>
@@ -124,18 +649,12 @@
     <t>09:17</t>
   </si>
   <si>
-    <t>07:50</t>
-  </si>
-  <si>
     <t>07:59</t>
   </si>
   <si>
     <t>08:36</t>
   </si>
   <si>
-    <t>08:51</t>
-  </si>
-  <si>
     <t>09:07</t>
   </si>
   <si>
@@ -148,36 +667,18 @@
     <t>09:52</t>
   </si>
   <si>
-    <t>10:12</t>
-  </si>
-  <si>
     <t>08:39</t>
   </si>
   <si>
-    <t>09:16</t>
-  </si>
-  <si>
     <t>09:31</t>
   </si>
   <si>
-    <t>09:47</t>
-  </si>
-  <si>
     <t>10:05</t>
   </si>
   <si>
-    <t>10:32</t>
-  </si>
-  <si>
     <t>10:52</t>
   </si>
   <si>
-    <t>09:10</t>
-  </si>
-  <si>
-    <t>09:19</t>
-  </si>
-  <si>
     <t>09:56</t>
   </si>
   <si>
@@ -199,9 +700,6 @@
     <t>10:15</t>
   </si>
   <si>
-    <t>10:24</t>
-  </si>
-  <si>
     <t>11:01</t>
   </si>
   <si>
@@ -277,9 +775,6 @@
     <t>13:36</t>
   </si>
   <si>
-    <t>13:52</t>
-  </si>
-  <si>
     <t>14:10</t>
   </si>
   <si>
@@ -301,12 +796,6 @@
     <t>14:11</t>
   </si>
   <si>
-    <t>14:26</t>
-  </si>
-  <si>
-    <t>14:42</t>
-  </si>
-  <si>
     <t>15:00</t>
   </si>
   <si>
@@ -355,9 +844,6 @@
     <t>15:51</t>
   </si>
   <si>
-    <t>16:06</t>
-  </si>
-  <si>
     <t>16:40</t>
   </si>
   <si>
@@ -379,9 +865,6 @@
     <t>16:56</t>
   </si>
   <si>
-    <t>17:12</t>
-  </si>
-  <si>
     <t>17:30</t>
   </si>
   <si>
@@ -418,9 +901,6 @@
     <t>18:32</t>
   </si>
   <si>
-    <t>18:52</t>
-  </si>
-  <si>
     <t>17:10</t>
   </si>
   <si>
@@ -448,12 +928,6 @@
     <t>17:45</t>
   </si>
   <si>
-    <t>17:54</t>
-  </si>
-  <si>
-    <t>18:31</t>
-  </si>
-  <si>
     <t>18:46</t>
   </si>
   <si>
@@ -466,9 +940,6 @@
     <t>19:27</t>
   </si>
   <si>
-    <t>19:47</t>
-  </si>
-  <si>
     <t>20:07</t>
   </si>
   <si>
@@ -508,9 +979,6 @@
     <t>19:56</t>
   </si>
   <si>
-    <t>20:11</t>
-  </si>
-  <si>
     <t>20:27</t>
   </si>
   <si>
@@ -529,15 +997,9 @@
     <t>20:20</t>
   </si>
   <si>
-    <t>20:29</t>
-  </si>
-  <si>
     <t>21:06</t>
   </si>
   <si>
-    <t>21:21</t>
-  </si>
-  <si>
     <t>21:37</t>
   </si>
   <si>
@@ -550,9 +1012,6 @@
     <t>21:47</t>
   </si>
   <si>
-    <t>22:24</t>
-  </si>
-  <si>
     <t>22:39</t>
   </si>
   <si>
@@ -562,9 +1021,6 @@
     <t>23:13</t>
   </si>
   <si>
-    <t>101번</t>
-  </si>
-  <si>
     <t xml:space="preserve">  공항-제주버스터미널-동광양-천수동-오현중·고등학교-화북남문-삼양초등학교-신촌초등학교-조천리사무소-함덕고등학교-함덕해수욕장-김녕초등학교-월정리-용암해수단지-세화리-세화고등학교-성산고등학교-성산항입구-성산일출봉입구-고성리(구.한국물류)-신산리-표선리제주은행-남원읍사무소</t>
   </si>
   <si>
@@ -572,462 +1028,6 @@
   </si>
   <si>
     <t>첫차(성산일출봉 출발) 6:05, 막차 21:38, 배차간격 30분~120분, 금남여객(064-753-4423)</t>
-  </si>
-  <si>
-    <t>(시행일 : 2024.8.15.)</t>
-  </si>
-  <si>
-    <t>06:00</t>
-  </si>
-  <si>
-    <t>06:18</t>
-  </si>
-  <si>
-    <t>06:36</t>
-  </si>
-  <si>
-    <t>06:50</t>
-  </si>
-  <si>
-    <t>07:26</t>
-  </si>
-  <si>
-    <t>07:34</t>
-  </si>
-  <si>
-    <t>07:00</t>
-  </si>
-  <si>
-    <t>07:18</t>
-  </si>
-  <si>
-    <t>07:36</t>
-  </si>
-  <si>
-    <t>08:26</t>
-  </si>
-  <si>
-    <t>08:34</t>
-  </si>
-  <si>
-    <t>07:09</t>
-  </si>
-  <si>
-    <t>08:11</t>
-  </si>
-  <si>
-    <t>08:29</t>
-  </si>
-  <si>
-    <t>08:43</t>
-  </si>
-  <si>
-    <t>09:27</t>
-  </si>
-  <si>
-    <t>08:14</t>
-  </si>
-  <si>
-    <t>08:31</t>
-  </si>
-  <si>
-    <t>08:58</t>
-  </si>
-  <si>
-    <t>09:34</t>
-  </si>
-  <si>
-    <t>09:48</t>
-  </si>
-  <si>
-    <t>09:54</t>
-  </si>
-  <si>
-    <t>10:30</t>
-  </si>
-  <si>
-    <t>10:44</t>
-  </si>
-  <si>
-    <t>11:20</t>
-  </si>
-  <si>
-    <t>11:28</t>
-  </si>
-  <si>
-    <t>10:04</t>
-  </si>
-  <si>
-    <t>10:21</t>
-  </si>
-  <si>
-    <t>10:41</t>
-  </si>
-  <si>
-    <t>10:48</t>
-  </si>
-  <si>
-    <t>11:06</t>
-  </si>
-  <si>
-    <t>11:24</t>
-  </si>
-  <si>
-    <t>11:38</t>
-  </si>
-  <si>
-    <t>12:14</t>
-  </si>
-  <si>
-    <t>12:22</t>
-  </si>
-  <si>
-    <t>10:54</t>
-  </si>
-  <si>
-    <t>11:11</t>
-  </si>
-  <si>
-    <t>11:31</t>
-  </si>
-  <si>
-    <t>11:56</t>
-  </si>
-  <si>
-    <t>12:28</t>
-  </si>
-  <si>
-    <t>13:04</t>
-  </si>
-  <si>
-    <t>13:12</t>
-  </si>
-  <si>
-    <t>11:34</t>
-  </si>
-  <si>
-    <t>11:51</t>
-  </si>
-  <si>
-    <t>12:11</t>
-  </si>
-  <si>
-    <t>12:18</t>
-  </si>
-  <si>
-    <t>12:36</t>
-  </si>
-  <si>
-    <t>12:54</t>
-  </si>
-  <si>
-    <t>13:08</t>
-  </si>
-  <si>
-    <t>13:44</t>
-  </si>
-  <si>
-    <t>12:24</t>
-  </si>
-  <si>
-    <t>12:41</t>
-  </si>
-  <si>
-    <t>13:01</t>
-  </si>
-  <si>
-    <t>13:26</t>
-  </si>
-  <si>
-    <t>13:58</t>
-  </si>
-  <si>
-    <t>14:34</t>
-  </si>
-  <si>
-    <t>13:24</t>
-  </si>
-  <si>
-    <t>13:41</t>
-  </si>
-  <si>
-    <t>14:01</t>
-  </si>
-  <si>
-    <t>14:08</t>
-  </si>
-  <si>
-    <t>14:44</t>
-  </si>
-  <si>
-    <t>14:58</t>
-  </si>
-  <si>
-    <t>15:34</t>
-  </si>
-  <si>
-    <t>15:42</t>
-  </si>
-  <si>
-    <t>14:09</t>
-  </si>
-  <si>
-    <t>14:46</t>
-  </si>
-  <si>
-    <t>14:53</t>
-  </si>
-  <si>
-    <t>15:11</t>
-  </si>
-  <si>
-    <t>15:29</t>
-  </si>
-  <si>
-    <t>15:43</t>
-  </si>
-  <si>
-    <t>16:19</t>
-  </si>
-  <si>
-    <t>16:27</t>
-  </si>
-  <si>
-    <t>14:54</t>
-  </si>
-  <si>
-    <t>15:31</t>
-  </si>
-  <si>
-    <t>15:38</t>
-  </si>
-  <si>
-    <t>15:56</t>
-  </si>
-  <si>
-    <t>16:14</t>
-  </si>
-  <si>
-    <t>16:28</t>
-  </si>
-  <si>
-    <t>17:04</t>
-  </si>
-  <si>
-    <t>15:49</t>
-  </si>
-  <si>
-    <t>16:26</t>
-  </si>
-  <si>
-    <t>16:33</t>
-  </si>
-  <si>
-    <t>16:51</t>
-  </si>
-  <si>
-    <t>17:09</t>
-  </si>
-  <si>
-    <t>17:23</t>
-  </si>
-  <si>
-    <t>17:59</t>
-  </si>
-  <si>
-    <t>18:07</t>
-  </si>
-  <si>
-    <t>16:34</t>
-  </si>
-  <si>
-    <t>17:11</t>
-  </si>
-  <si>
-    <t>17:18</t>
-  </si>
-  <si>
-    <t>17:36</t>
-  </si>
-  <si>
-    <t>18:08</t>
-  </si>
-  <si>
-    <t>18:44</t>
-  </si>
-  <si>
-    <t>17:29</t>
-  </si>
-  <si>
-    <t>17:46</t>
-  </si>
-  <si>
-    <t>18:06</t>
-  </si>
-  <si>
-    <t>18:13</t>
-  </si>
-  <si>
-    <t>18:49</t>
-  </si>
-  <si>
-    <t>19:03</t>
-  </si>
-  <si>
-    <t>19:39</t>
-  </si>
-  <si>
-    <t>18:14</t>
-  </si>
-  <si>
-    <t>18:51</t>
-  </si>
-  <si>
-    <t>18:58</t>
-  </si>
-  <si>
-    <t>19:16</t>
-  </si>
-  <si>
-    <t>19:34</t>
-  </si>
-  <si>
-    <t>19:48</t>
-  </si>
-  <si>
-    <t>20:24</t>
-  </si>
-  <si>
-    <t>20:32</t>
-  </si>
-  <si>
-    <t>19:09</t>
-  </si>
-  <si>
-    <t>19:26</t>
-  </si>
-  <si>
-    <t>19:46</t>
-  </si>
-  <si>
-    <t>19:53</t>
-  </si>
-  <si>
-    <t>20:43</t>
-  </si>
-  <si>
-    <t>21:19</t>
-  </si>
-  <si>
-    <t>21:27</t>
-  </si>
-  <si>
-    <t>19:44</t>
-  </si>
-  <si>
-    <t>20:01</t>
-  </si>
-  <si>
-    <t>20:21</t>
-  </si>
-  <si>
-    <t>20:28</t>
-  </si>
-  <si>
-    <t>20:46</t>
-  </si>
-  <si>
-    <t>21:04</t>
-  </si>
-  <si>
-    <t>21:18</t>
-  </si>
-  <si>
-    <t>21:54</t>
-  </si>
-  <si>
-    <t>22:02</t>
-  </si>
-  <si>
-    <t>20:14</t>
-  </si>
-  <si>
-    <t>20:31</t>
-  </si>
-  <si>
-    <t>20:51</t>
-  </si>
-  <si>
-    <t>20:58</t>
-  </si>
-  <si>
-    <t>21:16</t>
-  </si>
-  <si>
-    <t>21:34</t>
-  </si>
-  <si>
-    <t>21:48</t>
-  </si>
-  <si>
-    <t>22:32</t>
-  </si>
-  <si>
-    <t>20:44</t>
-  </si>
-  <si>
-    <t>21:01</t>
-  </si>
-  <si>
-    <t>21:28</t>
-  </si>
-  <si>
-    <t>21:46</t>
-  </si>
-  <si>
-    <t>22:04</t>
-  </si>
-  <si>
-    <t>22:18</t>
-  </si>
-  <si>
-    <t>22:54</t>
-  </si>
-  <si>
-    <t>23:02</t>
-  </si>
-  <si>
-    <t>21:14</t>
-  </si>
-  <si>
-    <t>21:31</t>
-  </si>
-  <si>
-    <t>21:51</t>
-  </si>
-  <si>
-    <t>21:58</t>
-  </si>
-  <si>
-    <t>21:44</t>
-  </si>
-  <si>
-    <t>22:01</t>
-  </si>
-  <si>
-    <t>22:21</t>
-  </si>
-  <si>
-    <t>22:28</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 남원읍사무소-표선리사무소-신산리-고성리-성산일출봉입구-성산항입구-성산고등학교-세화고등학교-세화리-용암해수단지-월정리-김녕초등학교-함덕해수욕장-함덕고등학교-조천리사무소-신촌초등학교-삼양동주민센터-화북남문-오현중·고등학교-천수동-동광양-제주버스터미널-공항</t>
-  </si>
-  <si>
-    <t>남원 →일주동로 → 공항</t>
-  </si>
-  <si>
-    <t>첫차(성산일출봉 출발) 6:00, 막차 21:44, 배차간격 28분~43분, 금남여객(064-753-4423)</t>
   </si>
 </sst>
 </file>
@@ -1420,13 +1420,13 @@
   <sheetData>
     <row r="2" ht="100.0" customHeight="true">
       <c r="B2" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -1436,7 +1436,7 @@
     </row>
     <row r="3" ht="25.0" customHeight="true">
       <c r="B3" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1462,7 +1462,7 @@
     </row>
     <row r="5" ht="25.0" customHeight="true">
       <c r="B5" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
@@ -1472,7 +1472,7 @@
       <c r="H5"/>
       <c r="I5"/>
       <c r="J5" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K5"/>
     </row>
@@ -1534,22 +1534,22 @@
         <v>10</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" ht="40.0" customHeight="true">
@@ -1566,22 +1566,22 @@
         <v>10</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" ht="40.0" customHeight="true">
@@ -1589,31 +1589,31 @@
         <v>3.0</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" ht="40.0" customHeight="true">
@@ -1621,31 +1621,31 @@
         <v>4.0</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" ht="40.0" customHeight="true">
@@ -1653,31 +1653,31 @@
         <v>5.0</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" ht="40.0" customHeight="true">
@@ -1685,31 +1685,31 @@
         <v>6.0</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" ht="40.0" customHeight="true">
@@ -1717,31 +1717,31 @@
         <v>7.0</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E14" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="G14" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="G14" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>57</v>
-      </c>
       <c r="I14" s="12" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" ht="40.0" customHeight="true">
@@ -1749,31 +1749,31 @@
         <v>8.0</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" ht="40.0" customHeight="true">
@@ -1781,31 +1781,31 @@
         <v>9.0</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E16" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="G16" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="G16" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>72</v>
-      </c>
       <c r="I16" s="12" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" ht="40.0" customHeight="true">
@@ -1813,31 +1813,31 @@
         <v>10.0</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" ht="40.0" customHeight="true">
@@ -1845,31 +1845,31 @@
         <v>11.0</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>84</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" ht="40.0" customHeight="true">
@@ -1877,31 +1877,31 @@
         <v>12.0</v>
       </c>
       <c r="C19" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D19" s="12" t="s">
-        <v>93</v>
-      </c>
       <c r="E19" s="12" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I19" s="12" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" ht="40.0" customHeight="true">
@@ -1909,31 +1909,31 @@
         <v>13.0</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" ht="40.0" customHeight="true">
@@ -1941,31 +1941,31 @@
         <v>14.0</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="I21" s="12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="J21" s="12" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" ht="40.0" customHeight="true">
@@ -1973,31 +1973,31 @@
         <v>15.0</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="J22" s="12" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" ht="40.0" customHeight="true">
@@ -2005,31 +2005,31 @@
         <v>16.0</v>
       </c>
       <c r="C23" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="D23" s="12" t="s">
-        <v>127</v>
-      </c>
       <c r="E23" s="12" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="J23" s="12" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" ht="40.0" customHeight="true">
@@ -2037,31 +2037,31 @@
         <v>17.0</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J24" s="12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="K24" s="13" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" ht="40.0" customHeight="true">
@@ -2069,31 +2069,31 @@
         <v>18.0</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="J25" s="12" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="K25" s="13" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" ht="40.0" customHeight="true">
@@ -2101,31 +2101,31 @@
         <v>19.0</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="J26" s="12" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="K26" s="13" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="27" ht="40.0" customHeight="true">
@@ -2133,31 +2133,31 @@
         <v>20.0</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="I27" s="12" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="J27" s="12" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="K27" s="13" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" ht="40.0" customHeight="true">
@@ -2165,22 +2165,22 @@
         <v>21.0</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>174</v>
+        <v>10</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>175</v>
+        <v>10</v>
       </c>
       <c r="I28" s="12" t="s">
         <v>10</v>
@@ -2197,22 +2197,22 @@
         <v>22.0</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>180</v>
+        <v>10</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>181</v>
+        <v>10</v>
       </c>
       <c r="I29" s="15" t="s">
         <v>10</v>
@@ -2255,7 +2255,7 @@
   <sheetData>
     <row r="2" ht="100.0" customHeight="true">
       <c r="B2" s="17" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -2307,7 +2307,7 @@
       <c r="H5"/>
       <c r="I5"/>
       <c r="J5" s="23" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K5"/>
     </row>
@@ -2369,22 +2369,22 @@
         <v>10</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>187</v>
+        <v>10</v>
       </c>
       <c r="G8" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="28" t="s">
         <v>188</v>
       </c>
-      <c r="H8" s="28" t="s">
+      <c r="I8" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="I8" s="28" t="s">
+      <c r="J8" s="28" t="s">
         <v>190</v>
       </c>
-      <c r="J8" s="28" t="s">
+      <c r="K8" s="29" t="s">
         <v>191</v>
-      </c>
-      <c r="K8" s="29" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="9" ht="40.0" customHeight="true">
@@ -2401,22 +2401,22 @@
         <v>10</v>
       </c>
       <c r="F9" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="I9" s="28" t="s">
         <v>193</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="J9" s="28" t="s">
         <v>194</v>
       </c>
-      <c r="H9" s="28" t="s">
+      <c r="K9" s="29" t="s">
         <v>195</v>
-      </c>
-      <c r="I9" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="J9" s="28" t="s">
-        <v>196</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="10" ht="40.0" customHeight="true">
@@ -2424,31 +2424,31 @@
         <v>3.0</v>
       </c>
       <c r="C10" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="E10" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="F10" s="28" t="s">
         <v>198</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>191</v>
-      </c>
-      <c r="E10" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="28" t="s">
-        <v>24</v>
       </c>
       <c r="G10" s="28" t="s">
         <v>199</v>
       </c>
       <c r="H10" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="J10" s="28" t="s">
         <v>200</v>
       </c>
-      <c r="I10" s="28" t="s">
+      <c r="K10" s="29" t="s">
         <v>201</v>
-      </c>
-      <c r="J10" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="K10" s="29" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="11" ht="40.0" customHeight="true">
@@ -2456,31 +2456,31 @@
         <v>4.0</v>
       </c>
       <c r="C11" s="28" t="s">
+        <v>202</v>
+      </c>
+      <c r="D11" s="28" t="s">
         <v>203</v>
       </c>
-      <c r="D11" s="28" t="s">
+      <c r="E11" s="28" t="s">
         <v>204</v>
-      </c>
-      <c r="E11" s="28" t="s">
-        <v>39</v>
       </c>
       <c r="F11" s="28" t="s">
         <v>205</v>
       </c>
       <c r="G11" s="28" t="s">
-        <v>46</v>
+        <v>206</v>
       </c>
       <c r="H11" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>61</v>
+        <v>209</v>
       </c>
       <c r="K11" s="29" t="s">
-        <v>50</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" ht="40.0" customHeight="true">
@@ -2488,31 +2488,31 @@
         <v>5.0</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="E12" s="28" t="s">
-        <v>48</v>
+        <v>212</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>208</v>
+        <v>33</v>
       </c>
       <c r="G12" s="28" t="s">
-        <v>44</v>
+        <v>213</v>
       </c>
       <c r="H12" s="28" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I12" s="28" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="J12" s="28" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K12" s="29" t="s">
-        <v>212</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" ht="40.0" customHeight="true">
@@ -2520,31 +2520,31 @@
         <v>6.0</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="E13" s="28" t="s">
-        <v>215</v>
+        <v>35</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>217</v>
+        <v>41</v>
       </c>
       <c r="H13" s="28" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I13" s="28" t="s">
-        <v>219</v>
+        <v>43</v>
       </c>
       <c r="J13" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="K13" s="29" t="s">
         <v>220</v>
-      </c>
-      <c r="K13" s="29" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="14" ht="40.0" customHeight="true">
@@ -2552,31 +2552,31 @@
         <v>7.0</v>
       </c>
       <c r="C14" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>221</v>
+      </c>
+      <c r="F14" s="28" t="s">
         <v>222</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="G14" s="28" t="s">
         <v>223</v>
       </c>
-      <c r="E14" s="28" t="s">
+      <c r="H14" s="28" t="s">
         <v>224</v>
       </c>
-      <c r="F14" s="28" t="s">
-        <v>219</v>
-      </c>
-      <c r="G14" s="28" t="s">
+      <c r="I14" s="28" t="s">
+        <v>220</v>
+      </c>
+      <c r="J14" s="28" t="s">
         <v>225</v>
       </c>
-      <c r="H14" s="28" t="s">
-        <v>220</v>
-      </c>
-      <c r="I14" s="28" t="s">
+      <c r="K14" s="29" t="s">
         <v>226</v>
-      </c>
-      <c r="J14" s="28" t="s">
-        <v>227</v>
-      </c>
-      <c r="K14" s="29" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="15" ht="40.0" customHeight="true">
@@ -2584,31 +2584,31 @@
         <v>8.0</v>
       </c>
       <c r="C15" s="28" t="s">
+        <v>227</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="F15" s="28" t="s">
         <v>229</v>
       </c>
-      <c r="D15" s="28" t="s">
+      <c r="G15" s="28" t="s">
+        <v>226</v>
+      </c>
+      <c r="H15" s="28" t="s">
         <v>230</v>
       </c>
-      <c r="E15" s="28" t="s">
+      <c r="I15" s="28" t="s">
         <v>231</v>
       </c>
-      <c r="F15" s="28" t="s">
+      <c r="J15" s="28" t="s">
         <v>232</v>
       </c>
-      <c r="G15" s="28" t="s">
+      <c r="K15" s="29" t="s">
         <v>233</v>
-      </c>
-      <c r="H15" s="28" t="s">
-        <v>234</v>
-      </c>
-      <c r="I15" s="28" t="s">
-        <v>235</v>
-      </c>
-      <c r="J15" s="28" t="s">
-        <v>236</v>
-      </c>
-      <c r="K15" s="29" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="16" ht="40.0" customHeight="true">
@@ -2616,31 +2616,31 @@
         <v>9.0</v>
       </c>
       <c r="C16" s="28" t="s">
+        <v>234</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>235</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>236</v>
+      </c>
+      <c r="F16" s="28" t="s">
         <v>237</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="G16" s="28" t="s">
+        <v>232</v>
+      </c>
+      <c r="H16" s="28" t="s">
         <v>238</v>
       </c>
-      <c r="E16" s="28" t="s">
+      <c r="I16" s="28" t="s">
         <v>239</v>
       </c>
-      <c r="F16" s="28" t="s">
-        <v>235</v>
-      </c>
-      <c r="G16" s="28" t="s">
+      <c r="J16" s="28" t="s">
         <v>240</v>
       </c>
-      <c r="H16" s="28" t="s">
-        <v>236</v>
-      </c>
-      <c r="I16" s="28" t="s">
+      <c r="K16" s="29" t="s">
         <v>241</v>
-      </c>
-      <c r="J16" s="28" t="s">
-        <v>242</v>
-      </c>
-      <c r="K16" s="29" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="17" ht="40.0" customHeight="true">
@@ -2648,31 +2648,31 @@
         <v>10.0</v>
       </c>
       <c r="C17" s="28" t="s">
+        <v>242</v>
+      </c>
+      <c r="D17" s="28" t="s">
         <v>243</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="E17" s="28" t="s">
         <v>244</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="F17" s="28" t="s">
         <v>245</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="G17" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="H17" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="G17" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="H17" s="28" t="s">
+      <c r="I17" s="28" t="s">
         <v>247</v>
       </c>
-      <c r="I17" s="28" t="s">
+      <c r="J17" s="28" t="s">
         <v>248</v>
       </c>
-      <c r="J17" s="28" t="s">
+      <c r="K17" s="29" t="s">
         <v>249</v>
-      </c>
-      <c r="K17" s="29" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="18" ht="40.0" customHeight="true">
@@ -2680,31 +2680,31 @@
         <v>11.0</v>
       </c>
       <c r="C18" s="28" t="s">
+        <v>238</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>250</v>
+      </c>
+      <c r="E18" s="28" t="s">
         <v>251</v>
       </c>
-      <c r="D18" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="E18" s="28" t="s">
+      <c r="F18" s="28" t="s">
         <v>252</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="G18" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" s="28" t="s">
         <v>253</v>
       </c>
-      <c r="G18" s="28" t="s">
+      <c r="I18" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="J18" s="28" t="s">
         <v>255</v>
       </c>
-      <c r="I18" s="28" t="s">
+      <c r="K18" s="29" t="s">
         <v>256</v>
-      </c>
-      <c r="J18" s="28" t="s">
-        <v>257</v>
-      </c>
-      <c r="K18" s="29" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="19" ht="40.0" customHeight="true">
@@ -2712,31 +2712,31 @@
         <v>12.0</v>
       </c>
       <c r="C19" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>258</v>
+      </c>
+      <c r="E19" s="28" t="s">
         <v>259</v>
       </c>
-      <c r="D19" s="28" t="s">
-        <v>254</v>
-      </c>
-      <c r="E19" s="28" t="s">
+      <c r="F19" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="G19" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="H19" s="28" t="s">
         <v>260</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="I19" s="28" t="s">
         <v>261</v>
       </c>
-      <c r="G19" s="28" t="s">
+      <c r="J19" s="28" t="s">
         <v>262</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="K19" s="29" t="s">
         <v>263</v>
-      </c>
-      <c r="I19" s="28" t="s">
-        <v>264</v>
-      </c>
-      <c r="J19" s="28" t="s">
-        <v>265</v>
-      </c>
-      <c r="K19" s="29" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="20" ht="40.0" customHeight="true">
@@ -2744,31 +2744,31 @@
         <v>13.0</v>
       </c>
       <c r="C20" s="28" t="s">
+        <v>264</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>265</v>
+      </c>
+      <c r="E20" s="28" t="s">
         <v>266</v>
       </c>
-      <c r="D20" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="E20" s="28" t="s">
+      <c r="F20" s="28" t="s">
         <v>267</v>
       </c>
-      <c r="F20" s="28" t="s">
+      <c r="G20" s="28" t="s">
         <v>268</v>
       </c>
-      <c r="G20" s="28" t="s">
+      <c r="H20" s="28" t="s">
         <v>269</v>
       </c>
-      <c r="H20" s="28" t="s">
+      <c r="I20" s="28" t="s">
         <v>270</v>
       </c>
-      <c r="I20" s="28" t="s">
+      <c r="J20" s="28" t="s">
         <v>271</v>
       </c>
-      <c r="J20" s="28" t="s">
+      <c r="K20" s="29" t="s">
         <v>272</v>
-      </c>
-      <c r="K20" s="29" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="21" ht="40.0" customHeight="true">
@@ -2776,31 +2776,31 @@
         <v>14.0</v>
       </c>
       <c r="C21" s="28" t="s">
+        <v>273</v>
+      </c>
+      <c r="D21" s="28" t="s">
         <v>274</v>
-      </c>
-      <c r="D21" s="28" t="s">
-        <v>269</v>
       </c>
       <c r="E21" s="28" t="s">
         <v>275</v>
       </c>
       <c r="F21" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" s="28" t="s">
+        <v>271</v>
+      </c>
+      <c r="H21" s="28" t="s">
         <v>276</v>
       </c>
-      <c r="G21" s="28" t="s">
+      <c r="I21" s="28" t="s">
         <v>277</v>
       </c>
-      <c r="H21" s="28" t="s">
-        <v>144</v>
-      </c>
-      <c r="I21" s="28" t="s">
+      <c r="J21" s="28" t="s">
         <v>278</v>
       </c>
-      <c r="J21" s="28" t="s">
+      <c r="K21" s="29" t="s">
         <v>279</v>
-      </c>
-      <c r="K21" s="29" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" ht="40.0" customHeight="true">
@@ -2808,31 +2808,31 @@
         <v>15.0</v>
       </c>
       <c r="C22" s="28" t="s">
+        <v>269</v>
+      </c>
+      <c r="D22" s="28" t="s">
         <v>280</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="E22" s="28" t="s">
         <v>281</v>
       </c>
-      <c r="E22" s="28" t="s">
+      <c r="F22" s="28" t="s">
         <v>282</v>
       </c>
-      <c r="F22" s="28" t="s">
+      <c r="G22" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="H22" s="28" t="s">
         <v>283</v>
       </c>
-      <c r="G22" s="28" t="s">
-        <v>145</v>
-      </c>
-      <c r="H22" s="28" t="s">
+      <c r="I22" s="28" t="s">
         <v>284</v>
       </c>
-      <c r="I22" s="28" t="s">
+      <c r="J22" s="28" t="s">
         <v>285</v>
       </c>
-      <c r="J22" s="28" t="s">
+      <c r="K22" s="29" t="s">
         <v>286</v>
-      </c>
-      <c r="K22" s="29" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="23" ht="40.0" customHeight="true">
@@ -2843,28 +2843,28 @@
         <v>287</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>145</v>
+        <v>288</v>
       </c>
       <c r="E23" s="28" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F23" s="28" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G23" s="28" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H23" s="28" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I23" s="28" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J23" s="28" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K23" s="29" t="s">
-        <v>294</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" ht="40.0" customHeight="true">
@@ -2884,19 +2884,19 @@
         <v>298</v>
       </c>
       <c r="G24" s="28" t="s">
-        <v>164</v>
+        <v>299</v>
       </c>
       <c r="H24" s="28" t="s">
-        <v>171</v>
+        <v>300</v>
       </c>
       <c r="I24" s="28" t="s">
-        <v>299</v>
+        <v>121</v>
       </c>
       <c r="J24" s="28" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K24" s="29" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="25" ht="40.0" customHeight="true">
@@ -2904,31 +2904,31 @@
         <v>18.0</v>
       </c>
       <c r="C25" s="28" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>303</v>
+        <v>118</v>
       </c>
       <c r="E25" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="28" t="s">
         <v>304</v>
       </c>
-      <c r="F25" s="28" t="s">
+      <c r="G25" s="28" t="s">
         <v>305</v>
       </c>
-      <c r="G25" s="28" t="s">
+      <c r="H25" s="28" t="s">
         <v>306</v>
       </c>
-      <c r="H25" s="28" t="s">
+      <c r="I25" s="28" t="s">
         <v>307</v>
       </c>
-      <c r="I25" s="28" t="s">
+      <c r="J25" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="K25" s="29" t="s">
         <v>308</v>
-      </c>
-      <c r="J25" s="28" t="s">
-        <v>309</v>
-      </c>
-      <c r="K25" s="29" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="26" ht="40.0" customHeight="true">
@@ -2936,31 +2936,31 @@
         <v>19.0</v>
       </c>
       <c r="C26" s="28" t="s">
+        <v>309</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="E26" s="28" t="s">
         <v>311</v>
       </c>
-      <c r="D26" s="28" t="s">
+      <c r="F26" s="28" t="s">
         <v>312</v>
       </c>
-      <c r="E26" s="28" t="s">
+      <c r="G26" s="28" t="s">
         <v>313</v>
       </c>
-      <c r="F26" s="28" t="s">
+      <c r="H26" s="28" t="s">
         <v>314</v>
       </c>
-      <c r="G26" s="28" t="s">
+      <c r="I26" s="28" t="s">
         <v>315</v>
       </c>
-      <c r="H26" s="28" t="s">
+      <c r="J26" s="28" t="s">
         <v>316</v>
       </c>
-      <c r="I26" s="28" t="s">
+      <c r="K26" s="29" t="s">
         <v>317</v>
-      </c>
-      <c r="J26" s="28" t="s">
-        <v>178</v>
-      </c>
-      <c r="K26" s="29" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="27" ht="40.0" customHeight="true">
@@ -2968,31 +2968,31 @@
         <v>20.0</v>
       </c>
       <c r="C27" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="D27" s="28" t="s">
         <v>319</v>
       </c>
-      <c r="D27" s="28" t="s">
+      <c r="E27" s="28" t="s">
         <v>320</v>
       </c>
-      <c r="E27" s="28" t="s">
-        <v>173</v>
-      </c>
       <c r="F27" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="G27" s="28" t="s">
         <v>321</v>
       </c>
-      <c r="G27" s="28" t="s">
+      <c r="H27" s="28" t="s">
         <v>322</v>
       </c>
-      <c r="H27" s="28" t="s">
+      <c r="I27" s="28" t="s">
         <v>323</v>
       </c>
-      <c r="I27" s="28" t="s">
+      <c r="J27" s="28" t="s">
         <v>324</v>
       </c>
-      <c r="J27" s="28" t="s">
+      <c r="K27" s="29" t="s">
         <v>325</v>
-      </c>
-      <c r="K27" s="29" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="28" ht="40.0" customHeight="true">
@@ -3000,22 +3000,22 @@
         <v>21.0</v>
       </c>
       <c r="C28" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="E28" s="28" t="s">
         <v>327</v>
       </c>
-      <c r="D28" s="28" t="s">
+      <c r="F28" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="G28" s="28" t="s">
         <v>328</v>
       </c>
-      <c r="E28" s="28" t="s">
+      <c r="H28" s="28" t="s">
         <v>329</v>
-      </c>
-      <c r="F28" s="28" t="s">
-        <v>330</v>
-      </c>
-      <c r="G28" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="H28" s="28" t="s">
-        <v>10</v>
       </c>
       <c r="I28" s="28" t="s">
         <v>10</v>
@@ -3032,22 +3032,22 @@
         <v>22.0</v>
       </c>
       <c r="C29" s="31" t="s">
+        <v>330</v>
+      </c>
+      <c r="D29" s="31" t="s">
         <v>331</v>
       </c>
-      <c r="D29" s="31" t="s">
+      <c r="E29" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="F29" s="31" t="s">
         <v>332</v>
       </c>
-      <c r="E29" s="31" t="s">
+      <c r="G29" s="31" t="s">
         <v>333</v>
       </c>
-      <c r="F29" s="31" t="s">
+      <c r="H29" s="31" t="s">
         <v>334</v>
-      </c>
-      <c r="G29" s="31" t="s">
-        <v>10</v>
-      </c>
-      <c r="H29" s="31" t="s">
-        <v>10</v>
       </c>
       <c r="I29" s="31" t="s">
         <v>10</v>

</xml_diff>